<commit_message>
Update DUS YCOA mapping and Bilanz/GuV workbooks
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DUS/1000 FDG Bilanz und GuV 2025 15.01.2026 mit Verkn..xlsx
+++ b/DUS/1000 FDG Bilanz und GuV 2025 15.01.2026 mit Verkn..xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="41" documentId="8_{5C260F46-EC54-41AB-AAD4-FF88C4C7A07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75CE3084-BF23-4254-BC83-D7F42DD47CD9}"/>
   <bookViews>
-    <workbookView xWindow="16230" yWindow="3000" windowWidth="21810" windowHeight="14835" xr2:uid="{FC069E69-F70E-4BCF-9679-BED290F6F4ED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FC069E69-F70E-4BCF-9679-BED290F6F4ED}"/>
   </bookViews>
   <sheets>
     <sheet name="SAP-Auszug" sheetId="5" r:id="rId1"/>
@@ -29660,12 +29660,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a2bfb3d0-c17c-4c08-a360-202b8d58d547">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -29864,20 +29866,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a2bfb3d0-c17c-4c08-a360-202b8d58d547">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABAC1596-DFFB-452B-BD1F-0BCBDAF30A28}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6932ED4-10ED-4670-AD8A-FF09AF2912DB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="a2bfb3d0-c17c-4c08-a360-202b8d58d547"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -29902,18 +29911,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6932ED4-10ED-4670-AD8A-FF09AF2912DB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABAC1596-DFFB-452B-BD1F-0BCBDAF30A28}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="a2bfb3d0-c17c-4c08-a360-202b8d58d547"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update DUS mapping files, add LOH F2S workshop material and Temp documents
</commit_message>
<xml_diff>
--- a/DUS/1000 FDG Bilanz und GuV 2025 15.01.2026 mit Verkn..xlsx
+++ b/DUS/1000 FDG Bilanz und GuV 2025 15.01.2026 mit Verkn..xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="41" documentId="8_{5C260F46-EC54-41AB-AAD4-FF88C4C7A07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75CE3084-BF23-4254-BC83-D7F42DD47CD9}"/>
   <bookViews>
-    <workbookView xWindow="16230" yWindow="3000" windowWidth="21810" windowHeight="14835" xr2:uid="{FC069E69-F70E-4BCF-9679-BED290F6F4ED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FC069E69-F70E-4BCF-9679-BED290F6F4ED}"/>
   </bookViews>
   <sheets>
     <sheet name="SAP-Auszug" sheetId="5" r:id="rId1"/>
@@ -29660,12 +29660,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a2bfb3d0-c17c-4c08-a360-202b8d58d547">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -29864,20 +29866,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a2bfb3d0-c17c-4c08-a360-202b8d58d547">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABAC1596-DFFB-452B-BD1F-0BCBDAF30A28}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6932ED4-10ED-4670-AD8A-FF09AF2912DB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="a2bfb3d0-c17c-4c08-a360-202b8d58d547"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -29902,18 +29911,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6932ED4-10ED-4670-AD8A-FF09AF2912DB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABAC1596-DFFB-452B-BD1F-0BCBDAF30A28}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="6e67c487-0b8d-48c6-8af2-8c60c3f722a0"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="a2bfb3d0-c17c-4c08-a360-202b8d58d547"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>